<commit_message>
Add product categories, inventory sync spreadsheet, and Reports print.
Introduce default product categories (editable in Setup), replace Download
template with Download inventory (Status + Category columns), import only
new SKUs, rename Sales History to Reports, and add inventory list printing.

Co-authored-by: theprincesajjad <theprincesajjad@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/product_import_template.xlsx
+++ b/assets/product_import_template.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Inventory" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="How to use" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,14 +418,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -445,59 +448,123 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Qty</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>60000</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Dell Latitude Laptop</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>i5 16GB 512GB</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>2</v>
-      </c>
-      <c r="E2" t="n">
-        <v>699.99</v>
+      <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="G6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="G7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="G8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="G9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="G10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="G11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="G12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="G13" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Category" error="Pick a category from the list or type a new one" type="list">
+      <formula1>"Cell Phones,Laptops,Desktops,Monitors,Printers,Accessories,Other"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="100" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>How to keep inventory up to date</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>60001</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Laptop Case</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>15.6 inch</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>10</v>
-      </c>
-      <c r="E3" t="n">
-        <v>15</v>
+          <t>1. Rows marked Status = In inventory are already in Retail Invoice — Import skips them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2. Add new products on blank rows below. Always fill in SKU (required) and Product Name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>3. Leave Status blank (or type New) for new rows.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>4. Save the file, then in Products click Import spreadsheet — only new SKUs are added.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>5. Categories: Cell Phones, Laptops, Desktops, Monitors, Printers, Accessories, Other</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>